<commit_message>
Refactor analysis to 1-0 matrix format
</commit_message>
<xml_diff>
--- a/test-files/butircerdas-uji-salah-format.xlsx
+++ b/test-files/butircerdas-uji-salah-format.xlsx
@@ -2,8 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jawaban" sheetId="1" r:id="Rf4261840e6a0482f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kunci" sheetId="2" r:id="Re5570a8c4c204f9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriks" sheetId="1" r:id="R9482881169c14824"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -221,91 +220,42 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="2.75" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.75" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="4.5" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="1.6299999952316284" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="1.75" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="5.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="5.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="5.130000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>No</x:v>
+        <x:v>Nama</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>Peserta</x:v>
+        <x:v>Soal 1</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
-        <x:v>Kelas</x:v>
-      </x:c>
-      <x:c r="D1" s="3" t="str">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E1" s="3" t="str">
-        <x:v>2</x:v>
+        <x:v>Soal 2</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="4" t="n">
-        <x:v>1</x:v>
+      <x:c r="A2" s="4" t="str">
+        <x:v>Salah</x:v>
       </x:c>
       <x:c r="B2" s="4" t="str">
-        <x:v>Salah Header</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="C2" s="4" t="str">
-        <x:v>X A</x:v>
-      </x:c>
-      <x:c r="D2" s="4" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="E2" s="4" t="str">
         <x:v>B</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="4" t="n">
-        <x:v>2</x:v>
+      <x:c r="A3" s="4" t="str">
+        <x:v>Format</x:v>
       </x:c>
       <x:c r="B3" s="4" t="str">
-        <x:v>Format Rusak</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="C3" s="4" t="str">
-        <x:v>X A</x:v>
-      </x:c>
-      <x:c r="D3" s="4" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E3" s="4" t="str">
         <x:v>D</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="5.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="4.75" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>Nomor</x:v>
-      </x:c>
-      <x:c r="B1" s="3" t="str">
-        <x:v>Kunci</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="4" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B2" s="4" t="str">
-        <x:v>A</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>